<commit_message>
CI Reports [2026-06-29 17:46]: ActionQueue — Excel reports updated
</commit_message>
<xml_diff>
--- a/Test Execution Report_Git/Daily Reports/BugReport_29-Jun-2026.xlsx
+++ b/Test Execution Report_Git/Daily Reports/BugReport_29-Jun-2026.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S2"/>
+  <dimension ref="A1:S27"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -538,9 +538,1484 @@
         <v>Test Execution Report\Feature Reports\Login.xlsx</v>
       </c>
     </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B3" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C3" t="str">
+        <v>TC-AQ-001</v>
+      </c>
+      <c r="D3" t="str">
+        <v>TC-AQ-001 | Page loads with heading and pending items</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Auto</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Critical</v>
+      </c>
+      <c r="H3" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I3" t="str">
+        <v>BUG-ACTIONQUEUE-001</v>
+      </c>
+      <c r="J3" t="str">
+        <v>[FAIL] TC-AQ-001 | Page loads with heading and pending items</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Critical</v>
+      </c>
+      <c r="L3" t="str">
+        <v>P1</v>
+      </c>
+      <c r="M3" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N3" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O3" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P3" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-AQ-001</v>
+      </c>
+      <c r="Q3" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R3" t="str">
+        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('[role="group"]') to be visible</v>
+      </c>
+      <c r="S3" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B4" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C4" t="str">
+        <v>TC-AQ-002</v>
+      </c>
+      <c r="D4" t="str">
+        <v>TC-AQ-002 | Stat cards display all 4 metrics</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F4" t="str">
+        <v>API</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H4" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I4" t="str">
+        <v>BUG-ACTIONQUEUE-002</v>
+      </c>
+      <c r="J4" t="str">
+        <v>[FAIL] TC-AQ-002 | Stat cards display all 4 metrics</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L4" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M4" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N4" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O4" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P4" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-AQ-002</v>
+      </c>
+      <c r="Q4" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R4" t="str">
+        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('[role="group"]') to be visible</v>
+      </c>
+      <c r="S4" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B5" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C5" t="str">
+        <v>TC-AQ-003</v>
+      </c>
+      <c r="D5" t="str">
+        <v>TC-AQ-003 | Grid displays all 10 expected column headers</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F5" t="str">
+        <v>API</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H5" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I5" t="str">
+        <v>BUG-ACTIONQUEUE-003</v>
+      </c>
+      <c r="J5" t="str">
+        <v>[FAIL] TC-AQ-003 | Grid displays all 10 expected column headers</v>
+      </c>
+      <c r="K5" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L5" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M5" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N5" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O5" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P5" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-AQ-003</v>
+      </c>
+      <c r="Q5" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R5" t="str">
+        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('[role="group"]') to be visible</v>
+      </c>
+      <c r="S5" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B6" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C6" t="str">
+        <v>TC-AQ-012</v>
+      </c>
+      <c r="D6" t="str">
+        <v>TC-AQ-012 | Search filters grid to matching rows</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Auto</v>
+      </c>
+      <c r="G6" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H6" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I6" t="str">
+        <v>BUG-ACTIONQUEUE-004</v>
+      </c>
+      <c r="J6" t="str">
+        <v>[FAIL] TC-AQ-012 | Search filters grid to matching rows</v>
+      </c>
+      <c r="K6" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L6" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M6" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N6" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O6" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P6" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-AQ-012</v>
+      </c>
+      <c r="Q6" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R6" t="str">
+        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('[role="group"]') to be visible</v>
+      </c>
+      <c r="S6" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B7" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C7" t="str">
+        <v>TC-AQ-020</v>
+      </c>
+      <c r="D7" t="str">
+        <v>TC-AQ-020 | No-match search shows empty grid</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Unit</v>
+      </c>
+      <c r="G7" t="str">
+        <v>High</v>
+      </c>
+      <c r="H7" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I7" t="str">
+        <v>BUG-ACTIONQUEUE-005</v>
+      </c>
+      <c r="J7" t="str">
+        <v>[FAIL] TC-AQ-020 | No-match search shows empty grid</v>
+      </c>
+      <c r="K7" t="str">
+        <v>High</v>
+      </c>
+      <c r="L7" t="str">
+        <v>P2</v>
+      </c>
+      <c r="M7" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N7" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O7" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P7" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-AQ-020</v>
+      </c>
+      <c r="Q7" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R7" t="str">
+        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('[role="group"]') to be visible</v>
+      </c>
+      <c r="S7" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B8" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C8" t="str">
+        <v>TC-AQ-014</v>
+      </c>
+      <c r="D8" t="str">
+        <v>TC-AQ-014 | EXPORT button is visible and clickable</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Auto</v>
+      </c>
+      <c r="G8" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H8" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I8" t="str">
+        <v>BUG-ACTIONQUEUE-006</v>
+      </c>
+      <c r="J8" t="str">
+        <v>[FAIL] TC-AQ-014 | EXPORT button is visible and clickable</v>
+      </c>
+      <c r="K8" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L8" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M8" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N8" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O8" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P8" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-AQ-014</v>
+      </c>
+      <c r="Q8" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R8" t="str">
+        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('[role="group"]') to be visible</v>
+      </c>
+      <c r="S8" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B9" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C9" t="str">
+        <v>TC-AQ-015</v>
+      </c>
+      <c r="D9" t="str">
+        <v>TC-AQ-015 | Pagination shows correct format</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F9" t="str">
+        <v>API</v>
+      </c>
+      <c r="G9" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H9" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I9" t="str">
+        <v>BUG-ACTIONQUEUE-007</v>
+      </c>
+      <c r="J9" t="str">
+        <v>[FAIL] TC-AQ-015 | Pagination shows correct format</v>
+      </c>
+      <c r="K9" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L9" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M9" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N9" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O9" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P9" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-AQ-015</v>
+      </c>
+      <c r="Q9" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R9" t="str">
+        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('[role="group"]') to be visible</v>
+      </c>
+      <c r="S9" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B10" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C10" t="str">
+        <v>TC-AQ-004</v>
+      </c>
+      <c r="D10" t="str">
+        <v>TC-AQ-004 | Perform Action opens ActionQueueDetails page</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F10" t="str">
+        <v>API</v>
+      </c>
+      <c r="G10" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H10" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I10" t="str">
+        <v>BUG-ACTIONQUEUE-008</v>
+      </c>
+      <c r="J10" t="str">
+        <v>[FAIL] TC-AQ-004 | Perform Action opens ActionQueueDetails page</v>
+      </c>
+      <c r="K10" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L10" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M10" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N10" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O10" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P10" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-AQ-004</v>
+      </c>
+      <c r="Q10" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R10" t="str">
+        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('[role="group"]') to be visible</v>
+      </c>
+      <c r="S10" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B11" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C11" t="str">
+        <v>TC-AQ-005</v>
+      </c>
+      <c r="D11" t="str">
+        <v>TC-AQ-005 | Detail page displays all 5 information sections</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F11" t="str">
+        <v>API</v>
+      </c>
+      <c r="G11" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H11" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I11" t="str">
+        <v>BUG-ACTIONQUEUE-009</v>
+      </c>
+      <c r="J11" t="str">
+        <v>[FAIL] TC-AQ-005 | Detail page displays all 5 information sections</v>
+      </c>
+      <c r="K11" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L11" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M11" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N11" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O11" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P11" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-AQ-005</v>
+      </c>
+      <c r="Q11" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R11" t="str">
+        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+      </c>
+      <c r="S11" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B12" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C12" t="str">
+        <v>TC-AQ-026</v>
+      </c>
+      <c r="D12" t="str">
+        <v>TC-AQ-026 | TIMELINE button opens timeline view</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F12" t="str">
+        <v>API</v>
+      </c>
+      <c r="G12" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H12" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I12" t="str">
+        <v>BUG-ACTIONQUEUE-010</v>
+      </c>
+      <c r="J12" t="str">
+        <v>[FAIL] TC-AQ-026 | TIMELINE button opens timeline view</v>
+      </c>
+      <c r="K12" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L12" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M12" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N12" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O12" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P12" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-AQ-026</v>
+      </c>
+      <c r="Q12" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R12" t="str">
+        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+      </c>
+      <c r="S12" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B13" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C13" t="str">
+        <v>TC-AQ-006</v>
+      </c>
+      <c r="D13" t="str">
+        <v>TC-AQ-006 | APPROVE dialog opens with correct elements</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F13" t="str">
+        <v>API</v>
+      </c>
+      <c r="G13" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H13" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I13" t="str">
+        <v>BUG-ACTIONQUEUE-011</v>
+      </c>
+      <c r="J13" t="str">
+        <v>[FAIL] TC-AQ-006 | APPROVE dialog opens with correct elements</v>
+      </c>
+      <c r="K13" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L13" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M13" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N13" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O13" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P13" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-AQ-006</v>
+      </c>
+      <c r="Q13" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R13" t="str">
+        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+      </c>
+      <c r="S13" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B14" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C14" t="str">
+        <v>TC-AQ-007</v>
+      </c>
+      <c r="D14" t="str">
+        <v>TC-AQ-007 | APPROVE with valid remarks submits successfully</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F14" t="str">
+        <v>API</v>
+      </c>
+      <c r="G14" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H14" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I14" t="str">
+        <v>BUG-ACTIONQUEUE-012</v>
+      </c>
+      <c r="J14" t="str">
+        <v>[FAIL] TC-AQ-007 | APPROVE with valid remarks submits successfully</v>
+      </c>
+      <c r="K14" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L14" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M14" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N14" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O14" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P14" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-AQ-007</v>
+      </c>
+      <c r="Q14" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R14" t="str">
+        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+      </c>
+      <c r="S14" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B15" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C15" t="str">
+        <v>TC-AQ-010</v>
+      </c>
+      <c r="D15" t="str">
+        <v>TC-AQ-010 | Cancel APPROVE dismisses without submitting</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F15" t="str">
+        <v>API</v>
+      </c>
+      <c r="G15" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H15" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I15" t="str">
+        <v>BUG-ACTIONQUEUE-013</v>
+      </c>
+      <c r="J15" t="str">
+        <v>[FAIL] TC-AQ-010 | Cancel APPROVE dismisses without submitting</v>
+      </c>
+      <c r="K15" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L15" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M15" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N15" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O15" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P15" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-AQ-010</v>
+      </c>
+      <c r="Q15" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R15" t="str">
+        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+      </c>
+      <c r="S15" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B16" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C16" t="str">
+        <v>TC-AQ-016</v>
+      </c>
+      <c r="D16" t="str">
+        <v>TC-AQ-016 | APPROVE empty remarks shows validation error</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F16" t="str">
+        <v>Unit</v>
+      </c>
+      <c r="G16" t="str">
+        <v>High</v>
+      </c>
+      <c r="H16" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I16" t="str">
+        <v>BUG-ACTIONQUEUE-014</v>
+      </c>
+      <c r="J16" t="str">
+        <v>[FAIL] TC-AQ-016 | APPROVE empty remarks shows validation error</v>
+      </c>
+      <c r="K16" t="str">
+        <v>High</v>
+      </c>
+      <c r="L16" t="str">
+        <v>P2</v>
+      </c>
+      <c r="M16" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N16" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O16" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P16" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-AQ-016</v>
+      </c>
+      <c r="Q16" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R16" t="str">
+        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+      </c>
+      <c r="S16" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B17" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C17" t="str">
+        <v>TC-AQ-021</v>
+      </c>
+      <c r="D17" t="str">
+        <v>TC-AQ-021 | Single character remarks accepted</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F17" t="str">
+        <v>API</v>
+      </c>
+      <c r="G17" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H17" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I17" t="str">
+        <v>BUG-ACTIONQUEUE-015</v>
+      </c>
+      <c r="J17" t="str">
+        <v>[FAIL] TC-AQ-021 | Single character remarks accepted</v>
+      </c>
+      <c r="K17" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L17" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M17" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N17" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O17" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P17" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-AQ-021</v>
+      </c>
+      <c r="Q17" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R17" t="str">
+        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+      </c>
+      <c r="S17" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B18" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C18" t="str">
+        <v>TC-AQ-022</v>
+      </c>
+      <c r="D18" t="str">
+        <v>TC-AQ-022 | Max length remarks (1000 chars) handled</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Boundary</v>
+      </c>
+      <c r="F18" t="str">
+        <v>API</v>
+      </c>
+      <c r="G18" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="H18" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I18" t="str">
+        <v>BUG-ACTIONQUEUE-016</v>
+      </c>
+      <c r="J18" t="str">
+        <v>[FAIL] TC-AQ-022 | Max length remarks (1000 chars) handled</v>
+      </c>
+      <c r="K18" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="L18" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M18" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N18" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O18" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P18" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-AQ-022</v>
+      </c>
+      <c r="Q18" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R18" t="str">
+        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+      </c>
+      <c r="S18" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B19" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C19" t="str">
+        <v>TC-AQ-023</v>
+      </c>
+      <c r="D19" t="str">
+        <v>TC-AQ-023 | Whitespace-only remarks rejected</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Boundary</v>
+      </c>
+      <c r="F19" t="str">
+        <v>Unit</v>
+      </c>
+      <c r="G19" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="H19" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I19" t="str">
+        <v>BUG-ACTIONQUEUE-017</v>
+      </c>
+      <c r="J19" t="str">
+        <v>[FAIL] TC-AQ-023 | Whitespace-only remarks rejected</v>
+      </c>
+      <c r="K19" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="L19" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M19" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N19" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O19" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P19" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-AQ-023</v>
+      </c>
+      <c r="Q19" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R19" t="str">
+        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+      </c>
+      <c r="S19" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B20" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C20" t="str">
+        <v>TC-AQ-024</v>
+      </c>
+      <c r="D20" t="str">
+        <v>TC-AQ-024 | SQL injection in remarks is sanitized</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Security</v>
+      </c>
+      <c r="F20" t="str">
+        <v>API</v>
+      </c>
+      <c r="G20" t="str">
+        <v>High</v>
+      </c>
+      <c r="H20" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I20" t="str">
+        <v>BUG-ACTIONQUEUE-018</v>
+      </c>
+      <c r="J20" t="str">
+        <v>[FAIL] TC-AQ-024 | SQL injection in remarks is sanitized</v>
+      </c>
+      <c r="K20" t="str">
+        <v>High</v>
+      </c>
+      <c r="L20" t="str">
+        <v>P2</v>
+      </c>
+      <c r="M20" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N20" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O20" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P20" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-AQ-024</v>
+      </c>
+      <c r="Q20" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R20" t="str">
+        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+      </c>
+      <c r="S20" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B21" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C21" t="str">
+        <v>TC-AQ-025</v>
+      </c>
+      <c r="D21" t="str">
+        <v>TC-AQ-025 | XSS payload in remarks @security</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Security</v>
+      </c>
+      <c r="F21" t="str">
+        <v>API</v>
+      </c>
+      <c r="G21" t="str">
+        <v>High</v>
+      </c>
+      <c r="H21" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I21" t="str">
+        <v>BUG-ACTIONQUEUE-019</v>
+      </c>
+      <c r="J21" t="str">
+        <v>[FAIL] TC-AQ-025 | XSS payload in remarks @security</v>
+      </c>
+      <c r="K21" t="str">
+        <v>High</v>
+      </c>
+      <c r="L21" t="str">
+        <v>P2</v>
+      </c>
+      <c r="M21" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N21" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O21" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P21" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-AQ-025</v>
+      </c>
+      <c r="Q21" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R21" t="str">
+        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+      </c>
+      <c r="S21" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B22" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C22" t="str">
+        <v>TC-AQ-008</v>
+      </c>
+      <c r="D22" t="str">
+        <v>TC-AQ-008 | REOPEN dialog opens with correct elements</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F22" t="str">
+        <v>API</v>
+      </c>
+      <c r="G22" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H22" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I22" t="str">
+        <v>BUG-ACTIONQUEUE-020</v>
+      </c>
+      <c r="J22" t="str">
+        <v>[FAIL] TC-AQ-008 | REOPEN dialog opens with correct elements</v>
+      </c>
+      <c r="K22" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L22" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M22" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N22" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O22" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P22" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-AQ-008</v>
+      </c>
+      <c r="Q22" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R22" t="str">
+        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+      </c>
+      <c r="S22" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B23" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C23" t="str">
+        <v>TC-AQ-009</v>
+      </c>
+      <c r="D23" t="str">
+        <v>TC-AQ-009 | REOPEN with valid remarks submits successfully</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F23" t="str">
+        <v>API</v>
+      </c>
+      <c r="G23" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H23" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I23" t="str">
+        <v>BUG-ACTIONQUEUE-021</v>
+      </c>
+      <c r="J23" t="str">
+        <v>[FAIL] TC-AQ-009 | REOPEN with valid remarks submits successfully</v>
+      </c>
+      <c r="K23" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L23" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M23" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N23" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O23" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P23" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-AQ-009</v>
+      </c>
+      <c r="Q23" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R23" t="str">
+        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+      </c>
+      <c r="S23" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B24" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C24" t="str">
+        <v>TC-AQ-011</v>
+      </c>
+      <c r="D24" t="str">
+        <v>TC-AQ-011 | Cancel REOPEN dismisses without submitting</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F24" t="str">
+        <v>API</v>
+      </c>
+      <c r="G24" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H24" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I24" t="str">
+        <v>BUG-ACTIONQUEUE-022</v>
+      </c>
+      <c r="J24" t="str">
+        <v>[FAIL] TC-AQ-011 | Cancel REOPEN dismisses without submitting</v>
+      </c>
+      <c r="K24" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L24" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M24" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N24" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O24" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P24" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-AQ-011</v>
+      </c>
+      <c r="Q24" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R24" t="str">
+        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+      </c>
+      <c r="S24" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B25" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C25" t="str">
+        <v>TC-AQ-017</v>
+      </c>
+      <c r="D25" t="str">
+        <v>TC-AQ-017 | REOPEN empty remarks shows validation error</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F25" t="str">
+        <v>Unit</v>
+      </c>
+      <c r="G25" t="str">
+        <v>High</v>
+      </c>
+      <c r="H25" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I25" t="str">
+        <v>BUG-ACTIONQUEUE-023</v>
+      </c>
+      <c r="J25" t="str">
+        <v>[FAIL] TC-AQ-017 | REOPEN empty remarks shows validation error</v>
+      </c>
+      <c r="K25" t="str">
+        <v>High</v>
+      </c>
+      <c r="L25" t="str">
+        <v>P2</v>
+      </c>
+      <c r="M25" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N25" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O25" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P25" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-AQ-017</v>
+      </c>
+      <c r="Q25" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R25" t="str">
+        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+      </c>
+      <c r="S25" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B26" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C26" t="str">
+        <v>TC-AQ-013</v>
+      </c>
+      <c r="D26" t="str">
+        <v>TC-AQ-013 | BACK button navigates away from detail page</v>
+      </c>
+      <c r="E26" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F26" t="str">
+        <v>Auto</v>
+      </c>
+      <c r="G26" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H26" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I26" t="str">
+        <v>BUG-ACTIONQUEUE-024</v>
+      </c>
+      <c r="J26" t="str">
+        <v>[FAIL] TC-AQ-013 | BACK button navigates away from detail page</v>
+      </c>
+      <c r="K26" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L26" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M26" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N26" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O26" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P26" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-AQ-013</v>
+      </c>
+      <c r="Q26" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R26" t="str">
+        <v>TimeoutError: locator.waitFor: Timeout 10000ms exceeded. Call log: - waiting for locator('text=RESOLUTION DESK') to be visible</v>
+      </c>
+      <c r="S26" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B27" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C27" t="str">
+        <v>ActionQueue-passed-29 Jun 2026</v>
+      </c>
+      <c r="D27" t="str">
+        <v>2 TCs passed — ActionQueue (FAILs above)</v>
+      </c>
+      <c r="E27" t="str">
+        <v>Mixed</v>
+      </c>
+      <c r="F27" t="str">
+        <v>Mixed</v>
+      </c>
+      <c r="G27" t="str">
+        <v>Mixed</v>
+      </c>
+      <c r="H27" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="I27" t="str">
+        <v>—</v>
+      </c>
+      <c r="J27" t="str">
+        <v>2/26 TCs passed</v>
+      </c>
+      <c r="K27" t="str">
+        <v>—</v>
+      </c>
+      <c r="L27" t="str">
+        <v>—</v>
+      </c>
+      <c r="M27" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N27" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O27" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P27" t="str">
+        <v>Playwright run: tests/actionqueue.spec.js</v>
+      </c>
+      <c r="Q27" t="str">
+        <v>Assertions pass</v>
+      </c>
+      <c r="R27" t="str">
+        <v>2/26 PASS | 24 FAILs logged</v>
+      </c>
+      <c r="S27" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S2"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S27"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
CI Reports [2026-06-29 19:07]: ActionQueue — Excel reports updated
</commit_message>
<xml_diff>
--- a/Test Execution Report_Git/Daily Reports/BugReport_29-Jun-2026.xlsx
+++ b/Test Execution Report_Git/Daily Reports/BugReport_29-Jun-2026.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S27"/>
+  <dimension ref="A1:S28"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -2013,9 +2013,68 @@
         <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B28" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C28" t="str">
+        <v>TC-AQ-018</v>
+      </c>
+      <c r="D28" t="str">
+        <v>TC-AQ-018 | Non-existent ticket ID handled gracefully</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F28" t="str">
+        <v>API</v>
+      </c>
+      <c r="G28" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H28" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I28" t="str">
+        <v>BUG-ACTIONQUEUE-025</v>
+      </c>
+      <c r="J28" t="str">
+        <v>[FAIL] TC-AQ-018 | Non-existent ticket ID handled gracefully</v>
+      </c>
+      <c r="K28" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L28" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M28" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N28" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O28" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P28" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-AQ-018</v>
+      </c>
+      <c r="Q28" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R28" t="str">
+        <v>TypeError: url.includes is not a function</v>
+      </c>
+      <c r="S28" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S27"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S28"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Regression [Nightly 2026-06-29 20:17]: all — reports updated
</commit_message>
<xml_diff>
--- a/Test Execution Report_Git/Daily Reports/BugReport_29-Jun-2026.xlsx
+++ b/Test Execution Report_Git/Daily Reports/BugReport_29-Jun-2026.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:S28"/>
+  <dimension ref="A1:S62"/>
   <cols>
     <col min="1" max="1" width="13.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
@@ -2072,9 +2072,2015 @@
         <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B29" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C29" t="str">
+        <v>TC-TICKET-001</v>
+      </c>
+      <c r="D29" t="str">
+        <v>TC-TICKET-001 | Create Ticket page loads with all required fields</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F29" t="str">
+        <v>Auto</v>
+      </c>
+      <c r="G29" t="str">
+        <v>Critical</v>
+      </c>
+      <c r="H29" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I29" t="str">
+        <v>BUG-ACTIONQUEUE-026</v>
+      </c>
+      <c r="J29" t="str">
+        <v>[FAIL] TC-TICKET-001 | Create Ticket page loads with all required fields</v>
+      </c>
+      <c r="K29" t="str">
+        <v>Critical</v>
+      </c>
+      <c r="L29" t="str">
+        <v>P1</v>
+      </c>
+      <c r="M29" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N29" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O29" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P29" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-TICKET-001</v>
+      </c>
+      <c r="Q29" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R29" t="str">
+        <v>TimeoutError: page.waitForSelector: Timeout 15000ms exceeded. Call log: - waiting for locator('#btnHeaderSubmit') to be visible</v>
+      </c>
+      <c r="S29" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B30" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C30" t="str">
+        <v>TC-TICKET-002</v>
+      </c>
+      <c r="D30" t="str">
+        <v>TC-TICKET-002 | Project dropdown shows all available projects</v>
+      </c>
+      <c r="E30" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F30" t="str">
+        <v>API</v>
+      </c>
+      <c r="G30" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H30" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I30" t="str">
+        <v>BUG-ACTIONQUEUE-027</v>
+      </c>
+      <c r="J30" t="str">
+        <v>[FAIL] TC-TICKET-002 | Project dropdown shows all available projects</v>
+      </c>
+      <c r="K30" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L30" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M30" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N30" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O30" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P30" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-TICKET-002</v>
+      </c>
+      <c r="Q30" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R30" t="str">
+        <v>TimeoutError: page.waitForSelector: Timeout 15000ms exceeded. Call log: - waiting for locator('#btnHeaderSubmit') to be visible</v>
+      </c>
+      <c r="S30" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B31" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C31" t="str">
+        <v>TC-TICKET-003</v>
+      </c>
+      <c r="D31" t="str">
+        <v>TC-TICKET-003 | All 6 Ticket Type chips are visible</v>
+      </c>
+      <c r="E31" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F31" t="str">
+        <v>Auto</v>
+      </c>
+      <c r="G31" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H31" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I31" t="str">
+        <v>BUG-ACTIONQUEUE-028</v>
+      </c>
+      <c r="J31" t="str">
+        <v>[FAIL] TC-TICKET-003 | All 6 Ticket Type chips are visible</v>
+      </c>
+      <c r="K31" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L31" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M31" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N31" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O31" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P31" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-TICKET-003</v>
+      </c>
+      <c r="Q31" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R31" t="str">
+        <v>TimeoutError: page.waitForSelector: Timeout 15000ms exceeded. Call log: - waiting for locator('#btnHeaderSubmit') to be visible</v>
+      </c>
+      <c r="S31" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B32" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C32" t="str">
+        <v>TC-TICKET-004</v>
+      </c>
+      <c r="D32" t="str">
+        <v>TC-TICKET-004 | All 6 platform chips visible on page load</v>
+      </c>
+      <c r="E32" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F32" t="str">
+        <v>Auto</v>
+      </c>
+      <c r="G32" t="str">
+        <v>Critical</v>
+      </c>
+      <c r="H32" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I32" t="str">
+        <v>BUG-ACTIONQUEUE-029</v>
+      </c>
+      <c r="J32" t="str">
+        <v>[FAIL] TC-TICKET-004 | All 6 platform chips visible on page load</v>
+      </c>
+      <c r="K32" t="str">
+        <v>Critical</v>
+      </c>
+      <c r="L32" t="str">
+        <v>P1</v>
+      </c>
+      <c r="M32" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N32" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O32" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P32" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-TICKET-004</v>
+      </c>
+      <c r="Q32" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R32" t="str">
+        <v>TimeoutError: page.waitForSelector: Timeout 15000ms exceeded. Call log: - waiting for locator('#btnHeaderSubmit') to be visible</v>
+      </c>
+      <c r="S32" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B33" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C33" t="str">
+        <v>TC-TICKET-005</v>
+      </c>
+      <c r="D33" t="str">
+        <v>TC-TICKET-005 | Description character counter updates on input</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F33" t="str">
+        <v>API</v>
+      </c>
+      <c r="G33" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H33" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I33" t="str">
+        <v>BUG-ACTIONQUEUE-030</v>
+      </c>
+      <c r="J33" t="str">
+        <v>[FAIL] TC-TICKET-005 | Description character counter updates on input</v>
+      </c>
+      <c r="K33" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L33" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M33" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N33" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O33" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P33" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-TICKET-005</v>
+      </c>
+      <c r="Q33" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R33" t="str">
+        <v>TimeoutError: page.waitForSelector: Timeout 15000ms exceeded. Call log: - waiting for locator('#btnHeaderSubmit') to be visible</v>
+      </c>
+      <c r="S33" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B34" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C34" t="str">
+        <v>TC-TICKET-006</v>
+      </c>
+      <c r="D34" t="str">
+        <v>TC-TICKET-006 | File attachment — PNG upload accepted</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F34" t="str">
+        <v>API</v>
+      </c>
+      <c r="G34" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H34" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I34" t="str">
+        <v>BUG-ACTIONQUEUE-031</v>
+      </c>
+      <c r="J34" t="str">
+        <v>[FAIL] TC-TICKET-006 | File attachment — PNG upload accepted</v>
+      </c>
+      <c r="K34" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L34" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M34" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N34" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O34" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P34" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-TICKET-006</v>
+      </c>
+      <c r="Q34" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R34" t="str">
+        <v>TimeoutError: page.waitForSelector: Timeout 15000ms exceeded. Call log: - waiting for locator('#btnHeaderSubmit') to be visible</v>
+      </c>
+      <c r="S34" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B35" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C35" t="str">
+        <v>TC-TICKET-007</v>
+      </c>
+      <c r="D35" t="str">
+        <v>TC-TICKET-007 | Reset button clears all filled fields</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F35" t="str">
+        <v>API</v>
+      </c>
+      <c r="G35" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H35" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I35" t="str">
+        <v>BUG-ACTIONQUEUE-032</v>
+      </c>
+      <c r="J35" t="str">
+        <v>[FAIL] TC-TICKET-007 | Reset button clears all filled fields</v>
+      </c>
+      <c r="K35" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L35" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M35" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N35" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O35" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P35" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-TICKET-007</v>
+      </c>
+      <c r="Q35" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R35" t="str">
+        <v>TimeoutError: page.waitForSelector: Timeout 15000ms exceeded. Call log: - waiting for locator('#btnHeaderSubmit') to be visible</v>
+      </c>
+      <c r="S35" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B36" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C36" t="str">
+        <v>TC-TICKET-008</v>
+      </c>
+      <c r="D36" t="str">
+        <v>TC-TICKET-008 | Submit with no fields filled shows Missing Information</v>
+      </c>
+      <c r="E36" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F36" t="str">
+        <v>API</v>
+      </c>
+      <c r="G36" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H36" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I36" t="str">
+        <v>BUG-ACTIONQUEUE-033</v>
+      </c>
+      <c r="J36" t="str">
+        <v>[FAIL] TC-TICKET-008 | Submit with no fields filled shows Missing Information</v>
+      </c>
+      <c r="K36" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L36" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M36" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N36" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O36" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P36" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-TICKET-008</v>
+      </c>
+      <c r="Q36" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R36" t="str">
+        <v>TimeoutError: page.waitForSelector: Timeout 15000ms exceeded. Call log: - waiting for locator('#btnHeaderSubmit') to be visible</v>
+      </c>
+      <c r="S36" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B37" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C37" t="str">
+        <v>TC-TICKET-009</v>
+      </c>
+      <c r="D37" t="str">
+        <v>TC-TICKET-009 | Submit without Project shows validation error</v>
+      </c>
+      <c r="E37" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F37" t="str">
+        <v>API</v>
+      </c>
+      <c r="G37" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H37" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I37" t="str">
+        <v>BUG-ACTIONQUEUE-034</v>
+      </c>
+      <c r="J37" t="str">
+        <v>[FAIL] TC-TICKET-009 | Submit without Project shows validation error</v>
+      </c>
+      <c r="K37" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L37" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M37" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N37" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O37" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P37" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-TICKET-009</v>
+      </c>
+      <c r="Q37" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R37" t="str">
+        <v>TimeoutError: page.waitForSelector: Timeout 15000ms exceeded. Call log: - waiting for locator('#btnHeaderSubmit') to be visible</v>
+      </c>
+      <c r="S37" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B38" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C38" t="str">
+        <v>TC-TICKET-010</v>
+      </c>
+      <c r="D38" t="str">
+        <v>TC-TICKET-010 | Submit without Ticket Type shows validation error</v>
+      </c>
+      <c r="E38" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F38" t="str">
+        <v>API</v>
+      </c>
+      <c r="G38" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H38" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I38" t="str">
+        <v>BUG-ACTIONQUEUE-035</v>
+      </c>
+      <c r="J38" t="str">
+        <v>[FAIL] TC-TICKET-010 | Submit without Ticket Type shows validation error</v>
+      </c>
+      <c r="K38" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L38" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M38" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N38" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O38" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P38" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-TICKET-010</v>
+      </c>
+      <c r="Q38" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R38" t="str">
+        <v>TimeoutError: page.waitForSelector: Timeout 15000ms exceeded. Call log: - waiting for locator('#btnHeaderSubmit') to be visible</v>
+      </c>
+      <c r="S38" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B39" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C39" t="str">
+        <v>TC-TICKET-011</v>
+      </c>
+      <c r="D39" t="str">
+        <v>TC-TICKET-011 | Submit without Description shows validation error</v>
+      </c>
+      <c r="E39" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F39" t="str">
+        <v>API</v>
+      </c>
+      <c r="G39" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H39" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I39" t="str">
+        <v>BUG-ACTIONQUEUE-036</v>
+      </c>
+      <c r="J39" t="str">
+        <v>[FAIL] TC-TICKET-011 | Submit without Description shows validation error</v>
+      </c>
+      <c r="K39" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L39" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M39" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N39" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O39" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P39" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-TICKET-011</v>
+      </c>
+      <c r="Q39" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R39" t="str">
+        <v>TimeoutError: page.waitForSelector: Timeout 15000ms exceeded. Call log: - waiting for locator('#btnHeaderSubmit') to be visible</v>
+      </c>
+      <c r="S39" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B40" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C40" t="str">
+        <v>TC-TICKET-012</v>
+      </c>
+      <c r="D40" t="str">
+        <v>TC-TICKET-012 | Submit with description under 15 chars blocked</v>
+      </c>
+      <c r="E40" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F40" t="str">
+        <v>API</v>
+      </c>
+      <c r="G40" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H40" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I40" t="str">
+        <v>BUG-ACTIONQUEUE-037</v>
+      </c>
+      <c r="J40" t="str">
+        <v>[FAIL] TC-TICKET-012 | Submit with description under 15 chars blocked</v>
+      </c>
+      <c r="K40" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L40" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M40" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N40" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O40" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P40" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-TICKET-012</v>
+      </c>
+      <c r="Q40" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R40" t="str">
+        <v>TimeoutError: page.waitForSelector: Timeout 15000ms exceeded. Call log: - waiting for locator('#btnHeaderSubmit') to be visible</v>
+      </c>
+      <c r="S40" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B41" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C41" t="str">
+        <v>TC-TICKET-013</v>
+      </c>
+      <c r="D41" t="str">
+        <v>TC-TICKET-013 | Page/Screen Name field is optional</v>
+      </c>
+      <c r="E41" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F41" t="str">
+        <v>API</v>
+      </c>
+      <c r="G41" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H41" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I41" t="str">
+        <v>BUG-ACTIONQUEUE-038</v>
+      </c>
+      <c r="J41" t="str">
+        <v>[FAIL] TC-TICKET-013 | Page/Screen Name field is optional</v>
+      </c>
+      <c r="K41" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L41" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M41" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N41" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O41" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P41" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-TICKET-013</v>
+      </c>
+      <c r="Q41" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R41" t="str">
+        <v>TimeoutError: page.waitForSelector: Timeout 15000ms exceeded. Call log: - waiting for locator('#btnHeaderSubmit') to be visible</v>
+      </c>
+      <c r="S41" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B42" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C42" t="str">
+        <v>TC-TICKET-014</v>
+      </c>
+      <c r="D42" t="str">
+        <v>TC-TICKET-014 | Description with exactly 15 chars passes validation</v>
+      </c>
+      <c r="E42" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F42" t="str">
+        <v>API</v>
+      </c>
+      <c r="G42" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H42" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I42" t="str">
+        <v>BUG-ACTIONQUEUE-039</v>
+      </c>
+      <c r="J42" t="str">
+        <v>[FAIL] TC-TICKET-014 | Description with exactly 15 chars passes validation</v>
+      </c>
+      <c r="K42" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L42" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M42" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N42" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O42" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P42" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-TICKET-014</v>
+      </c>
+      <c r="Q42" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R42" t="str">
+        <v>TimeoutError: page.waitForSelector: Timeout 15000ms exceeded. Call log: - waiting for locator('#btnHeaderSubmit') to be visible</v>
+      </c>
+      <c r="S42" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B43" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C43" t="str">
+        <v>TC-TICKET-015</v>
+      </c>
+      <c r="D43" t="str">
+        <v>TC-TICKET-015 | Description at 2000 chars accepted by counter</v>
+      </c>
+      <c r="E43" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F43" t="str">
+        <v>API</v>
+      </c>
+      <c r="G43" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H43" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I43" t="str">
+        <v>BUG-ACTIONQUEUE-040</v>
+      </c>
+      <c r="J43" t="str">
+        <v>[FAIL] TC-TICKET-015 | Description at 2000 chars accepted by counter</v>
+      </c>
+      <c r="K43" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L43" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M43" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N43" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O43" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P43" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-TICKET-015</v>
+      </c>
+      <c r="Q43" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R43" t="str">
+        <v>TimeoutError: page.waitForSelector: Timeout 15000ms exceeded. Call log: - waiting for locator('#btnHeaderSubmit') to be visible</v>
+      </c>
+      <c r="S43" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B44" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C44" t="str">
+        <v>TC-TICKET-016</v>
+      </c>
+      <c r="D44" t="str">
+        <v>TC-TICKET-016 | Description over 2000 chars truncated to max</v>
+      </c>
+      <c r="E44" t="str">
+        <v>Boundary</v>
+      </c>
+      <c r="F44" t="str">
+        <v>API</v>
+      </c>
+      <c r="G44" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="H44" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I44" t="str">
+        <v>BUG-ACTIONQUEUE-041</v>
+      </c>
+      <c r="J44" t="str">
+        <v>[FAIL] TC-TICKET-016 | Description over 2000 chars truncated to max</v>
+      </c>
+      <c r="K44" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="L44" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M44" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N44" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O44" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P44" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-TICKET-016</v>
+      </c>
+      <c r="Q44" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R44" t="str">
+        <v>TimeoutError: page.waitForSelector: Timeout 15000ms exceeded. Call log: - waiting for locator('#btnHeaderSubmit') to be visible</v>
+      </c>
+      <c r="S44" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B45" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C45" t="str">
+        <v>TC-TICKET-017</v>
+      </c>
+      <c r="D45" t="str">
+        <v>TC-TICKET-017 | Long page name (300 chars) handled gracefully</v>
+      </c>
+      <c r="E45" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F45" t="str">
+        <v>API</v>
+      </c>
+      <c r="G45" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H45" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I45" t="str">
+        <v>BUG-ACTIONQUEUE-042</v>
+      </c>
+      <c r="J45" t="str">
+        <v>[FAIL] TC-TICKET-017 | Long page name (300 chars) handled gracefully</v>
+      </c>
+      <c r="K45" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L45" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M45" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N45" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O45" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P45" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-TICKET-017</v>
+      </c>
+      <c r="Q45" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R45" t="str">
+        <v>TimeoutError: page.waitForSelector: Timeout 15000ms exceeded. Call log: - waiting for locator('#btnHeaderSubmit') to be visible</v>
+      </c>
+      <c r="S45" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B46" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C46" t="str">
+        <v>TC-TICKET-018</v>
+      </c>
+      <c r="D46" t="str">
+        <v>TC-TICKET-018 | Special characters in description handled safely</v>
+      </c>
+      <c r="E46" t="str">
+        <v>Boundary</v>
+      </c>
+      <c r="F46" t="str">
+        <v>API</v>
+      </c>
+      <c r="G46" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="H46" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I46" t="str">
+        <v>BUG-ACTIONQUEUE-043</v>
+      </c>
+      <c r="J46" t="str">
+        <v>[FAIL] TC-TICKET-018 | Special characters in description handled safely</v>
+      </c>
+      <c r="K46" t="str">
+        <v>Medium</v>
+      </c>
+      <c r="L46" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M46" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N46" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O46" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P46" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-TICKET-018</v>
+      </c>
+      <c r="Q46" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R46" t="str">
+        <v>TimeoutError: page.waitForSelector: Timeout 15000ms exceeded. Call log: - waiting for locator('#btnHeaderSubmit') to be visible</v>
+      </c>
+      <c r="S46" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B47" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C47" t="str">
+        <v>TC-TICKET-019</v>
+      </c>
+      <c r="D47" t="str">
+        <v>TC-TICKET-019 | SQL injection in description handled safely</v>
+      </c>
+      <c r="E47" t="str">
+        <v>Security</v>
+      </c>
+      <c r="F47" t="str">
+        <v>API</v>
+      </c>
+      <c r="G47" t="str">
+        <v>High</v>
+      </c>
+      <c r="H47" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I47" t="str">
+        <v>BUG-ACTIONQUEUE-044</v>
+      </c>
+      <c r="J47" t="str">
+        <v>[FAIL] TC-TICKET-019 | SQL injection in description handled safely</v>
+      </c>
+      <c r="K47" t="str">
+        <v>High</v>
+      </c>
+      <c r="L47" t="str">
+        <v>P2</v>
+      </c>
+      <c r="M47" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N47" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O47" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P47" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-TICKET-019</v>
+      </c>
+      <c r="Q47" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R47" t="str">
+        <v>TimeoutError: page.waitForSelector: Timeout 15000ms exceeded. Call log: - waiting for locator('#btnHeaderSubmit') to be visible</v>
+      </c>
+      <c r="S47" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B48" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C48" t="str">
+        <v>TC-TICKET-020</v>
+      </c>
+      <c r="D48" t="str">
+        <v>TC-TICKET-020 | XSS payload in description handled safely</v>
+      </c>
+      <c r="E48" t="str">
+        <v>Security</v>
+      </c>
+      <c r="F48" t="str">
+        <v>API</v>
+      </c>
+      <c r="G48" t="str">
+        <v>High</v>
+      </c>
+      <c r="H48" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I48" t="str">
+        <v>BUG-ACTIONQUEUE-045</v>
+      </c>
+      <c r="J48" t="str">
+        <v>[FAIL] TC-TICKET-020 | XSS payload in description handled safely</v>
+      </c>
+      <c r="K48" t="str">
+        <v>High</v>
+      </c>
+      <c r="L48" t="str">
+        <v>P2</v>
+      </c>
+      <c r="M48" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N48" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O48" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P48" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-TICKET-020</v>
+      </c>
+      <c r="Q48" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R48" t="str">
+        <v>TimeoutError: page.waitForSelector: Timeout 15000ms exceeded. Call log: - waiting for locator('#btnHeaderSubmit') to be visible</v>
+      </c>
+      <c r="S48" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B49" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C49" t="str">
+        <v>TC-TICKET-021</v>
+      </c>
+      <c r="D49" t="str">
+        <v>TC-TICKET-021 | Unauthenticated access redirected to login</v>
+      </c>
+      <c r="E49" t="str">
+        <v>Security</v>
+      </c>
+      <c r="F49" t="str">
+        <v>Auto</v>
+      </c>
+      <c r="G49" t="str">
+        <v>High</v>
+      </c>
+      <c r="H49" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I49" t="str">
+        <v>BUG-ACTIONQUEUE-046</v>
+      </c>
+      <c r="J49" t="str">
+        <v>[FAIL] TC-TICKET-021 | Unauthenticated access redirected to login</v>
+      </c>
+      <c r="K49" t="str">
+        <v>High</v>
+      </c>
+      <c r="L49" t="str">
+        <v>P2</v>
+      </c>
+      <c r="M49" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N49" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O49" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P49" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-TICKET-021</v>
+      </c>
+      <c r="Q49" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R49" t="str">
+        <v>TimeoutError: page.waitForSelector: Timeout 15000ms exceeded. Call log: - waiting for locator('#btnHeaderSubmit') to be visible</v>
+      </c>
+      <c r="S49" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B50" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C50" t="str">
+        <v>TC-TICKET-022</v>
+      </c>
+      <c r="D50" t="str">
+        <v>TC-TICKET-022 | HTML injection in description handled safely</v>
+      </c>
+      <c r="E50" t="str">
+        <v>Security</v>
+      </c>
+      <c r="F50" t="str">
+        <v>API</v>
+      </c>
+      <c r="G50" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H50" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I50" t="str">
+        <v>BUG-ACTIONQUEUE-047</v>
+      </c>
+      <c r="J50" t="str">
+        <v>[FAIL] TC-TICKET-022 | HTML injection in description handled safely</v>
+      </c>
+      <c r="K50" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L50" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M50" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N50" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O50" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P50" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-TICKET-022</v>
+      </c>
+      <c r="Q50" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R50" t="str">
+        <v>TimeoutError: page.waitForSelector: Timeout 15000ms exceeded. Call log: - waiting for locator('#btnHeaderSubmit') to be visible</v>
+      </c>
+      <c r="S50" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B51" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C51" t="str">
+        <v>TC-DASH-002</v>
+      </c>
+      <c r="D51" t="str">
+        <v>TC-DASH-002 | All 4 stat cards visible with values</v>
+      </c>
+      <c r="E51" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F51" t="str">
+        <v>Auto</v>
+      </c>
+      <c r="G51" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H51" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I51" t="str">
+        <v>BUG-ACTIONQUEUE-048</v>
+      </c>
+      <c r="J51" t="str">
+        <v>[FAIL] TC-DASH-002 | All 4 stat cards visible with values</v>
+      </c>
+      <c r="K51" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L51" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M51" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N51" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O51" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P51" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-DASH-002</v>
+      </c>
+      <c r="Q51" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R51" t="str">
+        <v>Error: expect(received).toBeTruthy() Received: false</v>
+      </c>
+      <c r="S51" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B52" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C52" t="str">
+        <v>TC-DASH-003</v>
+      </c>
+      <c r="D52" t="str">
+        <v>TC-DASH-003 | OVERVIEW and ANALYTICS buttons visible</v>
+      </c>
+      <c r="E52" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F52" t="str">
+        <v>Auto</v>
+      </c>
+      <c r="G52" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H52" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I52" t="str">
+        <v>BUG-ACTIONQUEUE-049</v>
+      </c>
+      <c r="J52" t="str">
+        <v>[FAIL] TC-DASH-003 | OVERVIEW and ANALYTICS buttons visible</v>
+      </c>
+      <c r="K52" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L52" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M52" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N52" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O52" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P52" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-DASH-003</v>
+      </c>
+      <c r="Q52" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R52" t="str">
+        <v>Error: expect(locator).toBeVisible() failed Locator: locator('#btnOverview') Expected: visible Timeout: 5000ms Error: element(s) not found Call log: - Expect "toBeVisible" with timeout 5000ms - waiting for locator('#btnOverview')</v>
+      </c>
+      <c r="S52" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B53" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C53" t="str">
+        <v>TC-DASH-004</v>
+      </c>
+      <c r="D53" t="str">
+        <v>TC-DASH-004 | ANALYTICS tab shows analytics content</v>
+      </c>
+      <c r="E53" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F53" t="str">
+        <v>Auto</v>
+      </c>
+      <c r="G53" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H53" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I53" t="str">
+        <v>BUG-ACTIONQUEUE-050</v>
+      </c>
+      <c r="J53" t="str">
+        <v>[FAIL] TC-DASH-004 | ANALYTICS tab shows analytics content</v>
+      </c>
+      <c r="K53" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L53" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M53" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N53" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O53" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P53" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-DASH-004</v>
+      </c>
+      <c r="Q53" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R53" t="str">
+        <v>Error: expect(received).toBeTruthy() Received: false</v>
+      </c>
+      <c r="S53" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B54" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C54" t="str">
+        <v>TC-DASH-005</v>
+      </c>
+      <c r="D54" t="str">
+        <v>TC-DASH-005 | Switch back to OVERVIEW from ANALYTICS</v>
+      </c>
+      <c r="E54" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F54" t="str">
+        <v>API</v>
+      </c>
+      <c r="G54" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H54" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I54" t="str">
+        <v>BUG-ACTIONQUEUE-051</v>
+      </c>
+      <c r="J54" t="str">
+        <v>[FAIL] TC-DASH-005 | Switch back to OVERVIEW from ANALYTICS</v>
+      </c>
+      <c r="K54" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L54" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M54" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N54" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O54" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P54" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-DASH-005</v>
+      </c>
+      <c r="Q54" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R54" t="str">
+        <v>Error: expect(received).toBeTruthy() Received: false</v>
+      </c>
+      <c r="S54" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B55" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C55" t="str">
+        <v>TC-DASH-006</v>
+      </c>
+      <c r="D55" t="str">
+        <v>TC-DASH-006 | Date range filter applies correctly</v>
+      </c>
+      <c r="E55" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F55" t="str">
+        <v>API</v>
+      </c>
+      <c r="G55" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H55" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I55" t="str">
+        <v>BUG-ACTIONQUEUE-052</v>
+      </c>
+      <c r="J55" t="str">
+        <v>[FAIL] TC-DASH-006 | Date range filter applies correctly</v>
+      </c>
+      <c r="K55" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L55" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M55" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N55" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O55" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P55" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-DASH-006</v>
+      </c>
+      <c r="Q55" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R55" t="str">
+        <v>TimeoutError: locator.fill: Timeout 15000ms exceeded. Call log: - waiting for locator('#dr_from') - locator resolved to &lt;input type="date" id="dr_from" max="2026-06-30" class="w-full text-[0.75rem] py-1.5 px-2 border border-gray-200 rounded mb-2 dark:bg-[#1a1a2e] dark:border-[#2b2b40] dark:text-gray</v>
+      </c>
+      <c r="S55" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B56" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C56" t="str">
+        <v>TC-DASH-007</v>
+      </c>
+      <c r="D56" t="str">
+        <v>TC-DASH-007 | Reset button clears date filter</v>
+      </c>
+      <c r="E56" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F56" t="str">
+        <v>API</v>
+      </c>
+      <c r="G56" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H56" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I56" t="str">
+        <v>BUG-ACTIONQUEUE-053</v>
+      </c>
+      <c r="J56" t="str">
+        <v>[FAIL] TC-DASH-007 | Reset button clears date filter</v>
+      </c>
+      <c r="K56" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L56" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M56" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N56" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O56" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P56" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-DASH-007</v>
+      </c>
+      <c r="Q56" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R56" t="str">
+        <v>TimeoutError: locator.fill: Timeout 15000ms exceeded. Call log: - waiting for locator('#dr_from') - locator resolved to &lt;input type="date" id="dr_from" max="2026-06-30" class="w-full text-[0.75rem] py-1.5 px-2 border border-gray-200 rounded mb-2 dark:bg-[#1a1a2e] dark:border-[#2b2b40] dark:text-gray</v>
+      </c>
+      <c r="S56" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B57" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C57" t="str">
+        <v>TC-DASH-008</v>
+      </c>
+      <c r="D57" t="str">
+        <v>TC-DASH-008 | Invalid date range To &lt; From handled gracefully</v>
+      </c>
+      <c r="E57" t="str">
+        <v>Negative</v>
+      </c>
+      <c r="F57" t="str">
+        <v>API</v>
+      </c>
+      <c r="G57" t="str">
+        <v>High</v>
+      </c>
+      <c r="H57" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I57" t="str">
+        <v>BUG-ACTIONQUEUE-054</v>
+      </c>
+      <c r="J57" t="str">
+        <v>[FAIL] TC-DASH-008 | Invalid date range To &lt; From handled gracefully</v>
+      </c>
+      <c r="K57" t="str">
+        <v>High</v>
+      </c>
+      <c r="L57" t="str">
+        <v>P2</v>
+      </c>
+      <c r="M57" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N57" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O57" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P57" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-DASH-008</v>
+      </c>
+      <c r="Q57" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R57" t="str">
+        <v>TimeoutError: locator.fill: Timeout 15000ms exceeded. Call log: - waiting for locator('#dr_from') - locator resolved to &lt;input type="date" id="dr_from" max="2026-06-30" class="w-full text-[0.75rem] py-1.5 px-2 border border-gray-200 rounded mb-2 dark:bg-[#1a1a2e] dark:border-[#2b2b40] dark:text-gray</v>
+      </c>
+      <c r="S57" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B58" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C58" t="str">
+        <v>TC-DASH-011</v>
+      </c>
+      <c r="D58" t="str">
+        <v>TC-DASH-011 | All sidebar navigation links present</v>
+      </c>
+      <c r="E58" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F58" t="str">
+        <v>API</v>
+      </c>
+      <c r="G58" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H58" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I58" t="str">
+        <v>BUG-ACTIONQUEUE-055</v>
+      </c>
+      <c r="J58" t="str">
+        <v>[FAIL] TC-DASH-011 | All sidebar navigation links present</v>
+      </c>
+      <c r="K58" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L58" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M58" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N58" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O58" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P58" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-DASH-011</v>
+      </c>
+      <c r="Q58" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R58" t="str">
+        <v>Error: expect(locator).toBeVisible() failed Locator: locator('a[href="/Ticket/Index"]').first() Expected: visible Received: hidden Timeout: 5000ms Call log: - Expect "toBeVisible" with timeout 5000ms - waiting for locator('a[href="/Ticket/Index"]').first() 14 × locator resolved to &lt;a data-id="4" tab</v>
+      </c>
+      <c r="S58" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B59" t="str">
+        <v>ActionQueue</v>
+      </c>
+      <c r="C59" t="str">
+        <v>TC-DASH-012</v>
+      </c>
+      <c r="D59" t="str">
+        <v>TC-DASH-012 | Action Queue badge shows ticket count</v>
+      </c>
+      <c r="E59" t="str">
+        <v>Positive</v>
+      </c>
+      <c r="F59" t="str">
+        <v>Auto</v>
+      </c>
+      <c r="G59" t="str">
+        <v>Low</v>
+      </c>
+      <c r="H59" t="str">
+        <v>FAIL</v>
+      </c>
+      <c r="I59" t="str">
+        <v>BUG-ACTIONQUEUE-056</v>
+      </c>
+      <c r="J59" t="str">
+        <v>[FAIL] TC-DASH-012 | Action Queue badge shows ticket count</v>
+      </c>
+      <c r="K59" t="str">
+        <v>Low</v>
+      </c>
+      <c r="L59" t="str">
+        <v>P3</v>
+      </c>
+      <c r="M59" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N59" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O59" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P59" t="str">
+        <v>See spec: tests/actionqueue.spec.js  TC: TC-DASH-012</v>
+      </c>
+      <c r="Q59" t="str">
+        <v>All Playwright assertions pass</v>
+      </c>
+      <c r="R59" t="str">
+        <v>Error: expect(received).toBeTruthy() Received: false</v>
+      </c>
+      <c r="S59" t="str">
+        <v>Test Execution Report\Feature Reports\ActionQueue.xlsx</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B60" t="str">
+        <v>CreateTicket</v>
+      </c>
+      <c r="C60" t="str">
+        <v>CreateTicket-passed-29 Jun 2026</v>
+      </c>
+      <c r="D60" t="str">
+        <v>27 TCs passed — CreateTicket (FAILs above)</v>
+      </c>
+      <c r="E60" t="str">
+        <v>Mixed</v>
+      </c>
+      <c r="F60" t="str">
+        <v>Mixed</v>
+      </c>
+      <c r="G60" t="str">
+        <v>Mixed</v>
+      </c>
+      <c r="H60" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="I60" t="str">
+        <v>—</v>
+      </c>
+      <c r="J60" t="str">
+        <v>27/83 TCs passed</v>
+      </c>
+      <c r="K60" t="str">
+        <v>—</v>
+      </c>
+      <c r="L60" t="str">
+        <v>—</v>
+      </c>
+      <c r="M60" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N60" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O60" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P60" t="str">
+        <v>Playwright run: tests/createticket.spec.js</v>
+      </c>
+      <c r="Q60" t="str">
+        <v>Assertions pass</v>
+      </c>
+      <c r="R60" t="str">
+        <v>27/83 PASS | 56 FAILs logged</v>
+      </c>
+      <c r="S60" t="str">
+        <v>Test Execution Report\Feature Reports\CreateTicket.xlsx</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B61" t="str">
+        <v>Dashboard</v>
+      </c>
+      <c r="C61" t="str">
+        <v>Dashboard-passed-29 Jun 2026</v>
+      </c>
+      <c r="D61" t="str">
+        <v>27 TCs passed — Dashboard (FAILs above)</v>
+      </c>
+      <c r="E61" t="str">
+        <v>Mixed</v>
+      </c>
+      <c r="F61" t="str">
+        <v>Mixed</v>
+      </c>
+      <c r="G61" t="str">
+        <v>Mixed</v>
+      </c>
+      <c r="H61" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="I61" t="str">
+        <v>—</v>
+      </c>
+      <c r="J61" t="str">
+        <v>27/83 TCs passed</v>
+      </c>
+      <c r="K61" t="str">
+        <v>—</v>
+      </c>
+      <c r="L61" t="str">
+        <v>—</v>
+      </c>
+      <c r="M61" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N61" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O61" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P61" t="str">
+        <v>Playwright run: tests/dashboard.spec.js</v>
+      </c>
+      <c r="Q61" t="str">
+        <v>Assertions pass</v>
+      </c>
+      <c r="R61" t="str">
+        <v>27/83 PASS | 56 FAILs logged</v>
+      </c>
+      <c r="S61" t="str">
+        <v>Test Execution Report\Feature Reports\Dashboard.xlsx</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="str">
+        <v>29 Jun 2026</v>
+      </c>
+      <c r="B62" t="str">
+        <v>Login</v>
+      </c>
+      <c r="C62" t="str">
+        <v>Login-passed-29 Jun 2026</v>
+      </c>
+      <c r="D62" t="str">
+        <v>27 TCs passed — Login (FAILs above)</v>
+      </c>
+      <c r="E62" t="str">
+        <v>Mixed</v>
+      </c>
+      <c r="F62" t="str">
+        <v>Mixed</v>
+      </c>
+      <c r="G62" t="str">
+        <v>Mixed</v>
+      </c>
+      <c r="H62" t="str">
+        <v>PASS</v>
+      </c>
+      <c r="I62" t="str">
+        <v>—</v>
+      </c>
+      <c r="J62" t="str">
+        <v>27/83 TCs passed</v>
+      </c>
+      <c r="K62" t="str">
+        <v>—</v>
+      </c>
+      <c r="L62" t="str">
+        <v>—</v>
+      </c>
+      <c r="M62" t="str">
+        <v>http://customerportal.dev-ts.online</v>
+      </c>
+      <c r="N62" t="str">
+        <v>Chrome</v>
+      </c>
+      <c r="O62" t="str">
+        <v>Windows</v>
+      </c>
+      <c r="P62" t="str">
+        <v>Playwright run: tests/login.spec.js</v>
+      </c>
+      <c r="Q62" t="str">
+        <v>Assertions pass</v>
+      </c>
+      <c r="R62" t="str">
+        <v>27/83 PASS | 56 FAILs logged</v>
+      </c>
+      <c r="S62" t="str">
+        <v>Test Execution Report\Feature Reports\Login.xlsx</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:S28"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:S62"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>